<commit_message>
update feature member management
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Clean Code</t>
   </si>
@@ -44,25 +44,13 @@
     <t>Kinh tế</t>
   </si>
   <si>
-    <t>Title</t>
-  </si>
-  <si>
-    <t>Author</t>
-  </si>
-  <si>
-    <t>Category</t>
-  </si>
-  <si>
-    <t>Quantity</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
     <t>Hướng dẫn các quy tắc và thực hành tốt nhất để viết mã nguồn sạch, dễ bảo trì cho lập trình viên.</t>
   </si>
   <si>
     <t>Đây là cuốn giáo khoa kinh tế học nổi tiếng nhất thế giới của Paul A. Samuelson và William D. Nordhaus, xuất bản lần đầu năm 1948 và đã được tái bản 15 lần, dịch ra nhiều thứ tiếng, được xem là chuẩn mực giảng dạy tại các trường đại học. Sách gồm 2 tập, tập 1 tập trung vào kinh tế học vi mô như cung cầu, thị trường sản phẩm và phân phối thu nhập, còn tập 2 nghiên cứu kinh tế vĩ mô gồm tổng cung, tăng trưởng kinh tế và thương mại quốc tế. Đây là tài liệu toàn diện và hệ thống, rất phù hợp cho sinh viên và người muốn tìm hiểu kinh tế học một cách căn bản.</t>
+  </si>
+  <si>
+    <t>CleanCode.png</t>
   </si>
 </sst>
 </file>
@@ -128,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -136,6 +124,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -416,31 +408,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.19921875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>10</v>
-      </c>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
     </row>
-    <row r="2" spans="1:5" ht="96.6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="69" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -451,13 +434,16 @@
         <v>2</v>
       </c>
       <c r="D2" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>11</v>
+        <v>6</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="409.6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" ht="358.8" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
@@ -471,8 +457,9 @@
         <v>3</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>12</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="F3" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
update the logic add barcode of bookCopies
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Clean Code</t>
   </si>
@@ -44,10 +44,28 @@
     <t>Kinh tế</t>
   </si>
   <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Author</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
     <t>Hướng dẫn các quy tắc và thực hành tốt nhất để viết mã nguồn sạch, dễ bảo trì cho lập trình viên.</t>
   </si>
   <si>
     <t>Đây là cuốn giáo khoa kinh tế học nổi tiếng nhất thế giới của Paul A. Samuelson và William D. Nordhaus, xuất bản lần đầu năm 1948 và đã được tái bản 15 lần, dịch ra nhiều thứ tiếng, được xem là chuẩn mực giảng dạy tại các trường đại học. Sách gồm 2 tập, tập 1 tập trung vào kinh tế học vi mô như cung cầu, thị trường sản phẩm và phân phối thu nhập, còn tập 2 nghiên cứu kinh tế vĩ mô gồm tổng cung, tăng trưởng kinh tế và thương mại quốc tế. Đây là tài liệu toàn diện và hệ thống, rất phù hợp cho sinh viên và người muốn tìm hiểu kinh tế học một cách căn bản.</t>
+  </si>
+  <si>
+    <t>imageUrl</t>
   </si>
   <si>
     <t>CleanCode.png</t>
@@ -416,12 +434,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
+      <c r="A1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="2" spans="1:6" ht="69" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -437,10 +467,10 @@
         <v>2</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="358.8" x14ac:dyDescent="0.25">
@@ -457,7 +487,7 @@
         <v>3</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="F3" s="4"/>
     </row>

</xml_diff>